<commit_message>
added inl to deployments
</commit_message>
<xml_diff>
--- a/notebooks/databases/MFRSR_History.xlsx
+++ b/notebooks/databases/MFRSR_History.xlsx
@@ -3,35 +3,36 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Overview" sheetId="1" r:id="rId3"/>
-    <sheet state="visible" name="451" sheetId="2" r:id="rId4"/>
-    <sheet state="visible" name="453" sheetId="3" r:id="rId5"/>
-    <sheet state="visible" name="607" sheetId="4" r:id="rId6"/>
-    <sheet state="visible" name="559" sheetId="5" r:id="rId7"/>
-    <sheet state="visible" name="584" sheetId="6" r:id="rId8"/>
-    <sheet state="visible" name="633" sheetId="7" r:id="rId9"/>
-    <sheet state="visible" name="632" sheetId="8" r:id="rId10"/>
-    <sheet state="visible" name="634" sheetId="9" r:id="rId11"/>
-    <sheet state="visible" name="635" sheetId="10" r:id="rId12"/>
-    <sheet state="visible" name="648" sheetId="11" r:id="rId13"/>
-    <sheet state="visible" name="649" sheetId="12" r:id="rId14"/>
-    <sheet state="visible" name="650" sheetId="13" r:id="rId15"/>
-    <sheet state="visible" name="651" sheetId="14" r:id="rId16"/>
-    <sheet state="visible" name="659" sheetId="15" r:id="rId17"/>
-    <sheet state="visible" name="660" sheetId="16" r:id="rId18"/>
-    <sheet state="visible" name="661" sheetId="17" r:id="rId19"/>
-    <sheet state="visible" name="662" sheetId="18" r:id="rId20"/>
-    <sheet state="visible" name="663" sheetId="19" r:id="rId21"/>
-    <sheet state="visible" name="664" sheetId="20" r:id="rId22"/>
-    <sheet state="visible" name="665" sheetId="21" r:id="rId23"/>
-    <sheet state="visible" name="669" sheetId="22" r:id="rId24"/>
-    <sheet state="visible" name="670" sheetId="23" r:id="rId25"/>
-    <sheet state="visible" name="671" sheetId="24" r:id="rId26"/>
-    <sheet state="visible" name="672" sheetId="25" r:id="rId27"/>
-    <sheet state="visible" name="673" sheetId="26" r:id="rId28"/>
-    <sheet state="visible" name="688" sheetId="27" r:id="rId29"/>
-    <sheet state="visible" name="689" sheetId="28" r:id="rId30"/>
-    <sheet state="visible" name="Notes" sheetId="29" r:id="rId31"/>
+    <sheet state="visible" name="Overview" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="451" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="453" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="607" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="559" sheetId="5" r:id="rId8"/>
+    <sheet state="visible" name="584" sheetId="6" r:id="rId9"/>
+    <sheet state="visible" name="633" sheetId="7" r:id="rId10"/>
+    <sheet state="visible" name="632" sheetId="8" r:id="rId11"/>
+    <sheet state="visible" name="634" sheetId="9" r:id="rId12"/>
+    <sheet state="visible" name="635" sheetId="10" r:id="rId13"/>
+    <sheet state="visible" name="648" sheetId="11" r:id="rId14"/>
+    <sheet state="visible" name="Sheet8" sheetId="12" r:id="rId15"/>
+    <sheet state="visible" name="649" sheetId="13" r:id="rId16"/>
+    <sheet state="visible" name="650" sheetId="14" r:id="rId17"/>
+    <sheet state="visible" name="651" sheetId="15" r:id="rId18"/>
+    <sheet state="visible" name="659" sheetId="16" r:id="rId19"/>
+    <sheet state="visible" name="660" sheetId="17" r:id="rId20"/>
+    <sheet state="visible" name="661" sheetId="18" r:id="rId21"/>
+    <sheet state="visible" name="662" sheetId="19" r:id="rId22"/>
+    <sheet state="visible" name="663" sheetId="20" r:id="rId23"/>
+    <sheet state="visible" name="664" sheetId="21" r:id="rId24"/>
+    <sheet state="visible" name="665" sheetId="22" r:id="rId25"/>
+    <sheet state="visible" name="669" sheetId="23" r:id="rId26"/>
+    <sheet state="visible" name="670" sheetId="24" r:id="rId27"/>
+    <sheet state="visible" name="671" sheetId="25" r:id="rId28"/>
+    <sheet state="visible" name="672" sheetId="26" r:id="rId29"/>
+    <sheet state="visible" name="673" sheetId="27" r:id="rId30"/>
+    <sheet state="visible" name="688" sheetId="28" r:id="rId31"/>
+    <sheet state="visible" name="689" sheetId="29" r:id="rId32"/>
+    <sheet state="visible" name="Notes" sheetId="30" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -41,16 +42,19 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={5af9e62f-a87f-4f00-a2fd-3bc89eae7088}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="F4">
+    <comment authorId="0" xr:uid="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}" ref="F4">
       <text>
-        <t xml:space="preserve">@Gary.Hodges@noaa.gov You mentioned below that this should be $AD23. is that correct? Why not just change it?
-_Assigned to Gary Hodges - NOAA Affiliate_
-	-Hagen Telg - NOAA Affiliate
-I just changed it.  Not sure why I didn't at the time???
-	-Gary Hodges - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	@gary.hodges@noaa.gov You mentioned below that this should be $AD23. is that correct? Why not just change it?
+Assigned to gary.hodges@noaa.gov
+Reply:
+	I just changed it.  Not sure why I didn't at the time???
+</t>
       </text>
     </comment>
   </commentList>
@@ -60,14 +64,17 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={afa8b239-4954-4803-8f0e-7fe2dbc39426}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="B11">
+    <comment authorId="0" xr:uid="{afa8b239-4954-4803-8f0e-7fe2dbc39426}" ref="N35">
       <text>
-        <t xml:space="preserve">@Gary.Hodges@noaa.gov should this read "present"?
-_Assigned to Gary Hodges - NOAA Affiliate_
-	-Hagen Telg - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	@gary.hodges@noaa.gov Is this correct?
+Assigned to gary.hodges@noaa.gov
+</t>
       </text>
     </comment>
   </commentList>
@@ -77,14 +84,17 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={474bdb03-b157-42c7-bd2d-54363d7a8a2a}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="B9">
+    <comment authorId="0" xr:uid="{474bdb03-b157-42c7-bd2d-54363d7a8a2a}" ref="B11">
       <text>
-        <t xml:space="preserve">@Gary.Hodges@noaa.gov should this read "present"?
-_Assigned to Gary Hodges - NOAA Affiliate_
-	-Hagen Telg - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	@gary.hodges@noaa.gov should this read "present"?
+Assigned to gary.hodges@noaa.gov
+</t>
       </text>
     </comment>
   </commentList>
@@ -94,19 +104,17 @@
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={a6eca3d6-12b0-4885-8774-5cee5686972a}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="C16">
+    <comment authorId="0" xr:uid="{a6eca3d6-12b0-4885-8774-5cee5686972a}" ref="B9">
       <text>
-        <t xml:space="preserve">is this right? I found this empty
-	-Hagen Telg - NOAA Affiliate</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="B16">
-      <text>
-        <t xml:space="preserve">is this right?
-	-Hagen Telg - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	@gary.hodges@noaa.gov should this read "present"?
+Assigned to gary.hodges@noaa.gov
+</t>
       </text>
     </comment>
   </commentList>
@@ -116,13 +124,28 @@
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={3e984a89-391f-4ad1-aa44-03eb9af178d6}</author>
+    <author>tc={949a4adf-7cc6-4586-b634-bfc5a0fb4cf7}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="A6">
+    <comment authorId="0" xr:uid="{3e984a89-391f-4ad1-aa44-03eb9af178d6}" ref="B16">
       <text>
-        <t xml:space="preserve">This is not the exact date! I just put this in in order to have a valid date format.
-	-Hagen Telg - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	is this right?
+Reply:
+	I have 665 as the MFR10 since 20191010.  What is the 20200310 date?
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{949a4adf-7cc6-4586-b634-bfc5a0fb4cf7}" ref="C16">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	is this right? I found this empty
+</t>
       </text>
     </comment>
   </commentList>
@@ -132,13 +155,37 @@
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author/>
+    <author>tc={4259c4e5-de2f-4b9e-9beb-146c5d668cd3}</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="A6">
+    <comment authorId="0" xr:uid="{4259c4e5-de2f-4b9e-9beb-146c5d668cd3}" ref="A6">
       <text>
-        <t xml:space="preserve">This is not the exact date! I just put this in in order to have a valid date format.
-	-Hagen Telg - NOAA Affiliate</t>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	This is not the exact date! I just put this in in order to have a valid date format.
+Reply:
+	688/689 were intended for Kettle Ponds but never went.  Went to Yankee for repair.  They finally sent them back a few weeks ago and FedEx lost the sensors.  Very sad to lose two new instruments.
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author>tc={ea2d1f94-e201-4456-a009-a99a41aaea9a}</author>
+  </authors>
+  <commentList>
+    <comment authorId="0" xr:uid="{ea2d1f94-e201-4456-a009-a99a41aaea9a}" ref="A6">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	This is not the exact date! I just put this in in order to have a valid date format.
+</t>
       </text>
     </comment>
   </commentList>
@@ -146,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="435">
   <si>
     <t>Instrument</t>
   </si>
@@ -1043,6 +1090,12 @@
     <t>Deploy to INL, Idaho Falls, ID site?</t>
   </si>
   <si>
+    <t>648/649</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
     <t>mfr649_20140110.xmd; mfr649_20140528.xmd</t>
   </si>
   <si>
@@ -1879,6 +1932,122 @@
 </styleSheet>
 </file>
 
+<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{b4e51d93-1f17-427b-b60b-a00675cbfc48}">
+    <Anchor>
+      <Comment id="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-01-16T16:47:37.00" id="{8ae39fe6-20f3-480f-8a18-a3a52c5e17c8}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-01-16T16:47:37.00" id="{f803cbd1-4e14-4bdb-bfee-a2ed77f3bf52}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}"/>
+        </Anchor>
+        <Assign userId="gary.hodges@noaa.gov" userName="gary.hodges@noaa.gov" userProvider="google-sheets"/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
+<file path=xl/documenttasks/documenttask2.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{fa62bb3c-428e-4a45-8a4e-037ce6d988df}">
+    <Anchor>
+      <Comment id="{afa8b239-4954-4803-8f0e-7fe2dbc39426}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-04-27T16:25:02.00" id="{5bae1622-bc49-4014-9e93-bf0ec4da8994}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{afa8b239-4954-4803-8f0e-7fe2dbc39426}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-04-27T16:25:02.00" id="{f77a5c2e-4ff4-4ab7-8ab4-e87b83354421}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{afa8b239-4954-4803-8f0e-7fe2dbc39426}"/>
+        </Anchor>
+        <Assign userId="gary.hodges@noaa.gov" userName="gary.hodges@noaa.gov" userProvider="google-sheets"/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
+<file path=xl/documenttasks/documenttask3.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{c0eefb88-fc2d-4e72-a568-39938444e14d}">
+    <Anchor>
+      <Comment id="{474bdb03-b157-42c7-bd2d-54363d7a8a2a}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-01-23T22:31:40.00" id="{5e43a10c-58fa-4d90-9b02-48c6fb0beed7}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{474bdb03-b157-42c7-bd2d-54363d7a8a2a}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-01-23T22:31:40.00" id="{e61052d6-13cb-49f6-923f-32a23f1e8810}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{474bdb03-b157-42c7-bd2d-54363d7a8a2a}"/>
+        </Anchor>
+        <Assign userId="gary.hodges@noaa.gov" userName="gary.hodges@noaa.gov" userProvider="google-sheets"/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
+<file path=xl/documenttasks/documenttask4.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{edc293a1-ade2-4ef1-845c-46d9adce9cca}">
+    <Anchor>
+      <Comment id="{a6eca3d6-12b0-4885-8774-5cee5686972a}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-01-23T22:31:27.00" id="{10301cec-7067-41d7-ab99-117fccfb51b7}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{a6eca3d6-12b0-4885-8774-5cee5686972a}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-01-23T22:31:27.00" id="{2677c772-50d4-48b2-ae30-30e9617cda96}">
+        <Attribution userId="placeholder@email.com" userName="Hagen Telg - NOAA Affiliate" userProvider="google-sheets"/>
+        <Anchor>
+          <Comment id="{a6eca3d6-12b0-4885-8774-5cee5686972a}"/>
+        </Anchor>
+        <Assign userId="gary.hodges@noaa.gov" userName="gary.hodges@noaa.gov" userProvider="google-sheets"/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
+<file path=xl/documenttasks/documenttask5.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
+</file>
+
+<file path=xl/documenttasks/documenttask6.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
+</file>
+
+<file path=xl/documenttasks/documenttask7.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -1971,6 +2140,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing30.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -1995,6 +2168,98 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <x18tc:person displayName="Hagen Telg - NOAA Affiliate" id="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" providerId="google-sheets"/>
+  <x18tc:person displayName="gary.hodges@noaa.gov" id="{4db97f81-caa7-4cfe-9c2f-adda9c0cf199}" userId="gary.hodges@noaa.gov" providerId="google-sheets"/>
+  <x18tc:person displayName="Gary Hodges - NOAA Affiliate" id="{4fa31c7b-fac6-4888-8c09-ecd10ef7ad00}" providerId="google-sheets"/>
+</x18tc:personList>
+</file>
+
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="F4" dT="2026-01-16T16:47:37.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}" done="0">
+    <x18tc:text xml:space="preserve">@gary.hodges@noaa.gov You mentioned below that this should be $AD23. is that correct? Why not just change it?
+Assigned to gary.hodges@noaa.gov</x18tc:text>
+    <x18tc:mentions>
+      <x18tc:mention mentionpersonId="{4db97f81-caa7-4cfe-9c2f-adda9c0cf199}" mentionId="{e2815d5c-38df-48c2-b99f-d41cfe0cd964}" startIndex="0" length="21"/>
+    </x18tc:mentions>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="F4" dT="2026-01-16T23:24:37.00" personId="{4fa31c7b-fac6-4888-8c09-ecd10ef7ad00}" id="{f6e7a4e6-fc9e-48df-84ea-c61d2dee589e}" parentId="{5af9e62f-a87f-4f00-a2fd-3bc89eae7088}">
+    <x18tc:text xml:space="preserve">I just changed it.  Not sure why I didn't at the time???</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="N35" dT="2026-04-27T16:25:02.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{afa8b239-4954-4803-8f0e-7fe2dbc39426}" done="1">
+    <x18tc:text xml:space="preserve">@gary.hodges@noaa.gov Is this correct?
+Assigned to gary.hodges@noaa.gov</x18tc:text>
+    <x18tc:mentions>
+      <x18tc:mention mentionpersonId="{4db97f81-caa7-4cfe-9c2f-adda9c0cf199}" mentionId="{cf04b067-2ce1-46b1-84b5-a16513bf3790}" startIndex="0" length="21"/>
+    </x18tc:mentions>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="B11" dT="2026-01-23T22:31:40.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{474bdb03-b157-42c7-bd2d-54363d7a8a2a}" done="1">
+    <x18tc:text xml:space="preserve">@gary.hodges@noaa.gov should this read "present"?
+Assigned to gary.hodges@noaa.gov</x18tc:text>
+    <x18tc:mentions>
+      <x18tc:mention mentionpersonId="{4db97f81-caa7-4cfe-9c2f-adda9c0cf199}" mentionId="{a5628f9d-5c64-472c-8236-7e592714af82}" startIndex="0" length="21"/>
+    </x18tc:mentions>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="B9" dT="2026-01-23T22:31:27.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{a6eca3d6-12b0-4885-8774-5cee5686972a}" done="1">
+    <x18tc:text xml:space="preserve">@gary.hodges@noaa.gov should this read "present"?
+Assigned to gary.hodges@noaa.gov</x18tc:text>
+    <x18tc:mentions>
+      <x18tc:mention mentionpersonId="{4db97f81-caa7-4cfe-9c2f-adda9c0cf199}" mentionId="{ef1ad515-8822-4a9a-8277-979431695cf1}" startIndex="0" length="21"/>
+    </x18tc:mentions>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment5.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="C16" dT="2026-01-27T23:59:26.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{949a4adf-7cc6-4586-b634-bfc5a0fb4cf7}" done="0">
+    <x18tc:text xml:space="preserve">is this right? I found this empty</x18tc:text>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="B16" dT="2026-01-27T23:59:08.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{3e984a89-391f-4ad1-aa44-03eb9af178d6}" done="0">
+    <x18tc:text xml:space="preserve">is this right?</x18tc:text>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="B16" dT="2026-04-28T20:04:26.00" personId="{4fa31c7b-fac6-4888-8c09-ecd10ef7ad00}" id="{6b109920-7458-43f5-818d-2f947aba7276}" parentId="{3e984a89-391f-4ad1-aa44-03eb9af178d6}">
+    <x18tc:text xml:space="preserve">I have 665 as the MFR10 since 20191010.  What is the 20200310 date?</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment6.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="A6" dT="2026-01-16T17:05:48.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{4259c4e5-de2f-4b9e-9beb-146c5d668cd3}" done="0">
+    <x18tc:text xml:space="preserve">This is not the exact date! I just put this in in order to have a valid date format.</x18tc:text>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="A6" dT="2026-04-28T20:05:51.00" personId="{4fa31c7b-fac6-4888-8c09-ecd10ef7ad00}" id="{f7016f6b-29d0-449f-ba35-d4f5eebd40d9}" parentId="{4259c4e5-de2f-4b9e-9beb-146c5d668cd3}">
+    <x18tc:text xml:space="preserve">688/689 were intended for Kettle Ponds but never went.  Went to Yankee for repair.  They finally sent them back a few weeks ago and FedEx lost the sensors.  Very sad to lose two new instruments.</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment7.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="A6" dT="2026-01-16T17:53:22.00" personId="{73bc003e-fed8-451b-a3b7-86bdeb2c2653}" id="{ea2d1f94-e201-4456-a009-a99a41aaea9a}" done="0">
+    <x18tc:text xml:space="preserve">This is not the exact date! I just put this in in order to have a valid date format.</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
@@ -2006,7 +2271,9 @@
     <col customWidth="1" min="1" max="6" width="10.56"/>
     <col customWidth="1" min="7" max="7" width="14.67"/>
     <col customWidth="1" min="8" max="9" width="18.56"/>
-    <col customWidth="1" min="10" max="15" width="10.56"/>
+    <col customWidth="1" min="10" max="10" width="10.56"/>
+    <col customWidth="1" min="11" max="11" width="13.67"/>
+    <col customWidth="1" min="12" max="15" width="10.56"/>
     <col customWidth="1" min="16" max="16" width="29.11"/>
     <col customWidth="1" min="17" max="27" width="10.56"/>
   </cols>
@@ -6322,8 +6589,8 @@
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup fitToHeight="0" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -10138,9 +10405,7 @@
       <c r="A23" s="70">
         <v>43900.0</v>
       </c>
-      <c r="B23" s="71" t="s">
-        <v>198</v>
-      </c>
+      <c r="B23" s="71"/>
       <c r="C23" s="45" t="s">
         <v>108</v>
       </c>
@@ -10345,7 +10610,7 @@
     </row>
     <row r="32">
       <c r="A32" s="75">
-        <v>45589.0</v>
+        <v>45246.0</v>
       </c>
       <c r="B32" s="75">
         <v>45950.0</v>
@@ -10401,8 +10666,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="69"/>
-      <c r="B35" s="69"/>
+      <c r="A35" s="70">
+        <v>46126.0</v>
+      </c>
+      <c r="B35" s="71" t="s">
+        <v>198</v>
+      </c>
       <c r="C35" s="44" t="s">
         <v>296</v>
       </c>
@@ -10418,11 +10687,13 @@
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
+      <c r="N35" s="44" t="s">
+        <v>298</v>
+      </c>
       <c r="O35" s="5"/>
     </row>
     <row r="36">
-      <c r="A36" s="69"/>
+      <c r="A36" s="58"/>
       <c r="B36" s="69"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -26912,11 +27183,29 @@
       <c r="O1005" s="5"/>
     </row>
   </sheetData>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="s">
+        <v>299</v>
+      </c>
+    </row>
+  </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -27071,7 +27360,7 @@
         <v>41</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>190</v>
@@ -27108,7 +27397,7 @@
         <v>42565.0</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
@@ -27266,7 +27555,7 @@
         <v>187</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
@@ -27345,7 +27634,7 @@
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="44" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -27370,7 +27659,7 @@
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="44" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16">
@@ -27394,7 +27683,7 @@
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="44" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="18">
@@ -27575,7 +27864,7 @@
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="44" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
@@ -27600,7 +27889,7 @@
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="44" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
@@ -30584,7 +30873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -30714,7 +31003,7 @@
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
       <c r="O3" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -30739,7 +31028,7 @@
         <v>41</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>190</v>
@@ -30754,7 +31043,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -30780,10 +31069,10 @@
       </c>
       <c r="D5" s="46"/>
       <c r="E5" s="46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="N5" s="46" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="6">
@@ -30812,7 +31101,7 @@
         <v>41</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E7" s="46" t="s">
         <v>15</v>
@@ -30830,7 +31119,7 @@
       </c>
       <c r="D8" s="46"/>
       <c r="E8" s="46" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -30844,13 +31133,13 @@
         <v>41</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E9" s="46" t="s">
         <v>15</v>
       </c>
       <c r="N9" s="46" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -30864,13 +31153,13 @@
         <v>108</v>
       </c>
       <c r="D10" s="46" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E10" s="46" t="s">
+        <v>316</v>
+      </c>
+      <c r="N10" s="46" t="s">
         <v>314</v>
-      </c>
-      <c r="N10" s="46" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="11">
@@ -30881,14 +31170,14 @@
         <v>198</v>
       </c>
       <c r="C11" s="54" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D11" s="46"/>
       <c r="E11" s="46" t="s">
         <v>17</v>
       </c>
       <c r="N11" s="46" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12">
@@ -33859,12 +34148,12 @@
       <c r="D1000" s="46"/>
     </row>
   </sheetData>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -33982,7 +34271,7 @@
         <v>261</v>
       </c>
       <c r="N3" s="46" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -33999,7 +34288,7 @@
         <v>17</v>
       </c>
       <c r="N4" s="46" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5">
@@ -34013,7 +34302,7 @@
         <v>108</v>
       </c>
       <c r="E5" s="46" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -34027,7 +34316,7 @@
         <v>41</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -34038,13 +34327,13 @@
         <v>42644.0</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E7" s="46" t="s">
         <v>15</v>
       </c>
       <c r="N7" s="46" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -34058,10 +34347,10 @@
         <v>108</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -34072,7 +34361,7 @@
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="O8" s="5"/>
     </row>
@@ -34084,22 +34373,22 @@
         <v>198</v>
       </c>
       <c r="C9" s="54" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E9" s="46" t="s">
         <v>17</v>
       </c>
       <c r="N9" s="46" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -34241,7 +34530,7 @@
         <v>42100.0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D4" s="50"/>
       <c r="E4" s="5" t="s">
@@ -34257,7 +34546,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -34298,7 +34587,7 @@
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="2"/>
@@ -34310,7 +34599,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="44" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7">
@@ -34362,7 +34651,7 @@
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
       <c r="O8" s="5" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -34377,7 +34666,7 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -34389,7 +34678,7 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
@@ -34414,11 +34703,11 @@
         <v>87</v>
       </c>
       <c r="E10" s="45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="N10" s="46"/>
       <c r="O10" s="45" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11">
@@ -34433,11 +34722,11 @@
       </c>
       <c r="D11" s="46"/>
       <c r="E11" s="54" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="N11" s="46"/>
       <c r="O11" s="54" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12">
@@ -34451,14 +34740,14 @@
         <v>162</v>
       </c>
       <c r="D12" s="46" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E12" s="46" t="s">
         <v>232</v>
       </c>
       <c r="N12" s="46"/>
       <c r="O12" s="46" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13">
@@ -34475,13 +34764,13 @@
         <v>187</v>
       </c>
       <c r="E13" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N13" s="46" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="O13" s="46" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -34526,7 +34815,7 @@
       </c>
       <c r="N15" s="46"/>
       <c r="O15" s="46" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16">
@@ -37516,7 +37805,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -37628,7 +37917,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -37668,7 +37957,7 @@
       </c>
       <c r="D4" s="50"/>
       <c r="E4" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="2"/>
@@ -37680,7 +37969,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -37706,7 +37995,7 @@
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
@@ -37743,7 +38032,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7">
@@ -37760,7 +38049,7 @@
         <v>232</v>
       </c>
       <c r="N7" s="46" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -37775,7 +38064,7 @@
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -37786,7 +38075,7 @@
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="O8" s="5"/>
     </row>
@@ -37804,7 +38093,7 @@
         <v>187</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
@@ -37815,7 +38104,7 @@
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="O9" s="5"/>
     </row>
@@ -37836,7 +38125,7 @@
         <v>17</v>
       </c>
       <c r="N10" s="46" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>
@@ -37844,7 +38133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -37956,7 +38245,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -37996,7 +38285,7 @@
       </c>
       <c r="D4" s="50"/>
       <c r="E4" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -38008,7 +38297,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -38034,7 +38323,7 @@
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
@@ -38071,7 +38360,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7">
@@ -38098,7 +38387,7 @@
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="8">
@@ -38115,7 +38404,7 @@
         <v>232</v>
       </c>
       <c r="N8" s="46" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -38130,7 +38419,7 @@
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
@@ -38141,7 +38430,7 @@
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="O9" s="5"/>
     </row>
@@ -38159,10 +38448,10 @@
         <v>187</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N10" s="46" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11">
@@ -38182,7 +38471,7 @@
         <v>17</v>
       </c>
       <c r="N11" s="46" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>
@@ -38190,7 +38479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -38302,7 +38591,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -38368,7 +38657,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6">
@@ -38383,7 +38672,7 @@
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -38395,7 +38684,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -38437,10 +38726,10 @@
         <v>232</v>
       </c>
       <c r="N8" s="54" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="O8" s="45" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9">
@@ -38457,10 +38746,10 @@
         <v>187</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N9" s="54" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -38471,13 +38760,13 @@
         <v>198</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>187</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -38488,10 +38777,10 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="54" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="O10" s="44" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
@@ -38510,22 +38799,22 @@
         <v>43748.0</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C11" s="45" t="s">
         <v>108</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="O11" s="45" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="90"/>
       <c r="O12" s="45" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13">
@@ -38536,11 +38825,11 @@
         <v>281</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="44" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
@@ -38561,11 +38850,11 @@
         <v>281</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="44" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -41541,7 +41830,39 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="s">
+        <v>176</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -41653,7 +41974,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -41692,10 +42013,10 @@
         <v>87</v>
       </c>
       <c r="E4" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5">
@@ -41712,7 +42033,7 @@
         <v>15</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6">
@@ -41727,7 +42048,7 @@
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="2"/>
@@ -41739,7 +42060,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -41768,7 +42089,7 @@
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -41779,7 +42100,7 @@
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="O8" s="5"/>
     </row>
@@ -41797,7 +42118,7 @@
         <v>232</v>
       </c>
       <c r="N9" s="46" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10">
@@ -41811,10 +42132,10 @@
         <v>26</v>
       </c>
       <c r="E10" s="46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="N10" s="46" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11">
@@ -41828,7 +42149,7 @@
         <v>26</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12">
@@ -41842,10 +42163,10 @@
         <v>108</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="O12" s="44" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13">
@@ -41856,11 +42177,11 @@
         <v>281</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="44" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
@@ -41881,11 +42202,11 @@
         <v>281</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="44" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
@@ -41903,39 +42224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="45" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="45" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="45" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="45" t="s">
-        <v>176</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -42047,7 +42336,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -42086,10 +42375,10 @@
         <v>154</v>
       </c>
       <c r="E4" s="46" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5">
@@ -42104,7 +42393,7 @@
       </c>
       <c r="D5" s="50"/>
       <c r="E5" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="2"/>
@@ -42116,7 +42405,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -42131,7 +42420,7 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
@@ -42168,7 +42457,7 @@
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8">
@@ -42185,7 +42474,7 @@
         <v>232</v>
       </c>
       <c r="N8" s="54" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9">
@@ -42202,7 +42491,7 @@
         <v>187</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -42213,11 +42502,11 @@
         <v>198</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -42228,10 +42517,10 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="44" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="O10" s="44" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
@@ -42253,16 +42542,16 @@
         <v>198</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="N11" s="45" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="O11" s="45" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -42270,7 +42559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -42382,7 +42671,7 @@
         <v>42100.0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D3" s="50"/>
       <c r="E3" s="5" t="s">
@@ -42421,10 +42710,10 @@
         <v>87</v>
       </c>
       <c r="E4" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N4" s="46" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="5">
@@ -42451,7 +42740,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6">
@@ -42466,7 +42755,7 @@
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="2"/>
@@ -42478,7 +42767,7 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -42545,7 +42834,7 @@
         <v>15</v>
       </c>
       <c r="O9" s="46" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -42560,7 +42849,7 @@
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -42571,7 +42860,7 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="O10" s="5"/>
     </row>
@@ -42589,7 +42878,7 @@
         <v>232</v>
       </c>
       <c r="N11" s="46" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="12">
@@ -42603,13 +42892,13 @@
         <v>26</v>
       </c>
       <c r="E12" s="46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="N12" s="46" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="O12" s="45" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="13">
@@ -42623,7 +42912,7 @@
         <v>26</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="14">
@@ -42637,7 +42926,7 @@
         <v>108</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
@@ -42645,19 +42934,19 @@
         <v>43748.0</v>
       </c>
       <c r="B15" s="45" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E15" s="45" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="N15" s="45" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="O15" s="45" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16">
@@ -42668,19 +42957,19 @@
         <v>198</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="O16" s="45" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -42816,7 +43105,7 @@
         <v>15</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5">
@@ -42834,7 +43123,7 @@
         <v>232</v>
       </c>
       <c r="N5" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6">
@@ -42848,13 +43137,13 @@
         <v>41</v>
       </c>
       <c r="D6" s="46" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N6" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -42872,7 +43161,7 @@
         <v>17</v>
       </c>
       <c r="N7" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8">
@@ -45859,7 +46148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -45998,7 +46287,7 @@
         <v>41</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E5" s="46" t="s">
         <v>15</v>
@@ -46019,7 +46308,7 @@
         <v>232</v>
       </c>
       <c r="N6" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7">
@@ -46033,13 +46322,13 @@
         <v>41</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N7" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -46057,7 +46346,7 @@
         <v>17</v>
       </c>
       <c r="N8" s="46" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9">
@@ -50034,7 +50323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -50172,7 +50461,7 @@
       </c>
       <c r="N4" s="46"/>
       <c r="O4" s="46" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5">
@@ -50201,7 +50490,7 @@
         <v>41</v>
       </c>
       <c r="D6" s="46" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E6" s="46" t="s">
         <v>232</v>
@@ -50222,7 +50511,7 @@
         <v>187</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -50234,7 +50523,7 @@
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -50273,11 +50562,11 @@
         <v>41</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="N9" s="46"/>
       <c r="O9" s="5" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="10">
@@ -50295,7 +50584,7 @@
       </c>
       <c r="N10" s="46"/>
       <c r="O10" s="46" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11">
@@ -54285,7 +54574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -54439,13 +54728,13 @@
         <v>41</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E5" s="46" t="s">
         <v>15</v>
       </c>
       <c r="N5" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6">
@@ -54462,10 +54751,10 @@
         <v>187</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N6" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7">
@@ -54479,16 +54768,16 @@
         <v>41</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N7" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="O7" s="46" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8">
@@ -54508,7 +54797,7 @@
         <v>15</v>
       </c>
       <c r="O8" s="46" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9">
@@ -54539,13 +54828,13 @@
         <v>162</v>
       </c>
       <c r="D10" s="46" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E10" s="46" t="s">
         <v>232</v>
       </c>
       <c r="N10" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="11">
@@ -54568,16 +54857,16 @@
         <v>260</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="O12" s="45" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -54585,7 +54874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -54708,7 +54997,7 @@
         <v>2</v>
       </c>
       <c r="N3" s="46" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4">
@@ -54722,13 +55011,13 @@
         <v>41</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E4" s="46" t="s">
         <v>15</v>
       </c>
       <c r="N4" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5">
@@ -54745,10 +55034,10 @@
         <v>187</v>
       </c>
       <c r="E5" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N5" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6">
@@ -54762,13 +55051,13 @@
         <v>41</v>
       </c>
       <c r="D6" s="46" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N6" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7">
@@ -54796,10 +55085,10 @@
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="8">
@@ -54819,7 +55108,7 @@
         <v>15</v>
       </c>
       <c r="N8" s="46" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9">
@@ -54833,7 +55122,7 @@
         <v>162</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>232</v>
@@ -54847,7 +55136,7 @@
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="O9" s="5"/>
     </row>
@@ -54879,7 +55168,7 @@
         <v>17</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12">
@@ -59829,146 +60118,6 @@
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D1" s="50" t="s">
-        <v>180</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="H1" s="2">
-        <v>415.0</v>
-      </c>
-      <c r="I1" s="2">
-        <v>500.0</v>
-      </c>
-      <c r="J1" s="2">
-        <v>1625.0</v>
-      </c>
-      <c r="K1" s="2">
-        <v>675.0</v>
-      </c>
-      <c r="L1" s="2">
-        <v>860.0</v>
-      </c>
-      <c r="M1" s="2">
-        <v>940.0</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="64">
-        <v>44545.0</v>
-      </c>
-      <c r="C2" s="45" t="s">
-        <v>393</v>
-      </c>
-      <c r="O2" s="45" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="56">
-        <v>44256.0</v>
-      </c>
-      <c r="B3" s="56">
-        <v>44270.0</v>
-      </c>
-      <c r="C3" s="45" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="45" t="s">
-        <v>395</v>
-      </c>
-      <c r="O3" s="94" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="E4" s="45" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="68"/>
-      <c r="B5" s="71" t="s">
-        <v>397</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>398</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="44" t="s">
-        <v>399</v>
-      </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="44" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="56">
-        <v>44409.0</v>
-      </c>
-      <c r="C6" s="45" t="s">
-        <v>154</v>
-      </c>
-      <c r="E6" s="45" t="s">
-        <v>401</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -60038,14 +60187,14 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="55">
-        <v>44180.0</v>
+      <c r="A2" s="64">
+        <v>44545.0</v>
       </c>
       <c r="C2" s="45" t="s">
-        <v>393</v>
-      </c>
-      <c r="O2" s="95" t="s">
-        <v>402</v>
+        <v>395</v>
+      </c>
+      <c r="O2" s="45" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="3">
@@ -60059,33 +60208,28 @@
         <v>108</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>395</v>
-      </c>
-      <c r="O3" s="96" t="s">
-        <v>403</v>
+        <v>397</v>
+      </c>
+      <c r="O3" s="94" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="4">
       <c r="E4" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="45" t="s">
-        <v>404</v>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="68">
-        <v>44470.0</v>
-      </c>
+      <c r="A5" s="68"/>
       <c r="B5" s="71" t="s">
-        <v>281</v>
+        <v>399</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="44" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
@@ -60096,7 +60240,9 @@
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
+      <c r="O5" s="44" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="56">
@@ -60106,12 +60252,12 @@
         <v>154</v>
       </c>
       <c r="E6" s="45" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -60123,161 +60269,138 @@
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H1" s="2">
+        <v>415.0</v>
+      </c>
+      <c r="I1" s="2">
+        <v>500.0</v>
+      </c>
+      <c r="J1" s="2">
+        <v>1625.0</v>
+      </c>
+      <c r="K1" s="2">
+        <v>675.0</v>
+      </c>
+      <c r="L1" s="2">
+        <v>860.0</v>
+      </c>
+      <c r="M1" s="2">
+        <v>940.0</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="55">
+        <v>44180.0</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>395</v>
+      </c>
+      <c r="O2" s="95" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="56">
+        <v>44256.0</v>
+      </c>
+      <c r="B3" s="56">
+        <v>44270.0</v>
+      </c>
+      <c r="C3" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" s="45" t="s">
+        <v>397</v>
+      </c>
+      <c r="O3" s="96" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="58" t="s">
+    <row r="4">
+      <c r="E4" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" s="45" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="97"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="58" t="s">
-        <v>407</v>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" s="97"/>
+      <c r="A5" s="68">
+        <v>44470.0</v>
+      </c>
+      <c r="B5" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="44" t="s">
+        <v>401</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="58" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="58" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="58" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="58" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="58" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="58" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="58" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="58" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="58" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="58" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="58" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="58" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="58" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="58" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="58" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="58" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="58" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="97"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="58" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="58" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="58" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="58" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="58" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="58" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="58" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="58" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="58" t="s">
-        <v>432</v>
+      <c r="A6" s="56">
+        <v>44409.0</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6" s="45" t="s">
+        <v>403</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -60289,7 +60412,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="3" width="10.56"/>
-    <col customWidth="1" min="4" max="4" width="28.89"/>
+    <col customWidth="1" min="4" max="4" width="36.33"/>
     <col customWidth="1" min="5" max="5" width="43.89"/>
     <col customWidth="1" min="6" max="26" width="10.56"/>
   </cols>
@@ -63437,6 +63560,172 @@
     </row>
     <row r="1000">
       <c r="D1000" s="46"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="58" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="58" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="97"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="58" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="97"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="58" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="58" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="58" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="58" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="58" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="58" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="58" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="58" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="58" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="58" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="58" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="58" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="58" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="58" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="58" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="58" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="58" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="97"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="58" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="58" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="58" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="58" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="58" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="58" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="58" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="58" t="s">
+        <v>434</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>